<commit_message>
Add NEDP review deck v3 in Bitwise style with updated STP/4P tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cx9kswyecF7JAB1Rr5vVcV
</commit_message>
<xml_diff>
--- a/nedp_deck/stp4p/Crane_STP_4P_Medium_Heavy.xlsx
+++ b/nedp_deck/stp4p/Crane_STP_4P_Medium_Heavy.xlsx
@@ -967,17 +967,17 @@
       </c>
       <c r="O5" s="37" t="inlineStr">
         <is>
-          <t>Italy-made; importer/dealer under assessment</t>
+          <t>Made in Europe</t>
         </is>
       </c>
       <c r="P5" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q5" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1032,8 +1032,7 @@
       </c>
       <c r="M6" s="43" t="inlineStr">
         <is>
-          <t>− Power boost (HPLS (MH), Top 1 only)
-− Extension speed (High speed ext. (ROU), Top 1 only)</t>
+          <t>Parity: wins on price/delivery</t>
         </is>
       </c>
       <c r="N6" s="45" t="n">
@@ -1041,17 +1040,17 @@
       </c>
       <c r="O6" s="37" t="inlineStr">
         <is>
-          <t>China-made; Palfinger Asia Pacific rep. office Jakarta, dealer network</t>
+          <t>Made in China</t>
         </is>
       </c>
       <c r="P6" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE mounting (partnership needed: GM Tractors holds XCMG); China-made</t>
+          <t>Negotiate special price with XCMG</t>
         </is>
       </c>
       <c r="Q6" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1106,8 +1105,7 @@
       </c>
       <c r="M7" s="40" t="inlineStr">
         <is>
-          <t>− Power boost (HPLS (MH), Top 1 only)
-− Extension speed (High speed ext. (ROU), Top 1 only)</t>
+          <t>Parity: wins on price/delivery</t>
         </is>
       </c>
       <c r="N7" s="42" t="n">
@@ -1115,17 +1113,17 @@
       </c>
       <c r="O7" s="37" t="inlineStr">
         <is>
-          <t>China-made; Palfinger Asia Pacific rep. office Jakarta, dealer network</t>
+          <t>Made in China</t>
         </is>
       </c>
       <c r="P7" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE mounting (partnership needed: GM Tractors holds XCMG); China-made</t>
+          <t>Negotiate special price with XCMG</t>
         </is>
       </c>
       <c r="Q7" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1192,17 +1190,17 @@
       </c>
       <c r="O8" s="37" t="inlineStr">
         <is>
-          <t>China-made; Palfinger Asia Pacific rep. office Jakarta, dealer network</t>
+          <t>Made in China</t>
         </is>
       </c>
       <c r="P8" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Negotiate price with Ferrari. Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q8" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1424,17 +1422,17 @@
       </c>
       <c r="O15" s="37" t="inlineStr">
         <is>
-          <t>Italy-made; importer/dealer under assessment</t>
+          <t>Made in Europe</t>
         </is>
       </c>
       <c r="P15" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q15" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1487,7 @@
       </c>
       <c r="M16" s="46" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Parity: wins on price/delivery</t>
         </is>
       </c>
       <c r="N16" s="48" t="n">
@@ -1497,17 +1495,17 @@
       </c>
       <c r="O16" s="37" t="inlineStr">
         <is>
-          <t>Austria-made; dealer PT Sanggar Sarana Baja (ABM Group) for mining</t>
+          <t>Made in Europe</t>
         </is>
       </c>
       <c r="P16" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Negotiate price with Ferrari. Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q16" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1578,17 +1576,17 @@
       </c>
       <c r="O17" s="37" t="inlineStr">
         <is>
-          <t>China-made; Palfinger Asia Pacific rep. office Jakarta, dealer network</t>
+          <t>Made in China</t>
         </is>
       </c>
       <c r="P17" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q17" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1641,7 @@
       </c>
       <c r="M18" s="46" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Parity: wins on price/delivery</t>
         </is>
       </c>
       <c r="N18" s="48" t="n">
@@ -1651,17 +1649,17 @@
       </c>
       <c r="O18" s="37" t="inlineStr">
         <is>
-          <t>Austria-made; dealer PT Sanggar Sarana Baja (ABM Group) for mining</t>
+          <t>Made in Europe</t>
         </is>
       </c>
       <c r="P18" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Negotiate price with Ferrari. Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q18" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1716,7 @@
       </c>
       <c r="M19" s="40" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>Parity: wins on price/delivery</t>
         </is>
       </c>
       <c r="N19" s="42" t="inlineStr">
@@ -1728,17 +1726,17 @@
       </c>
       <c r="O19" s="37" t="inlineStr">
         <is>
-          <t>Austria-made; dealer PT Sanggar Sarana Baja (ABM Group) for mining</t>
+          <t>Made in Europe</t>
         </is>
       </c>
       <c r="P19" s="37" t="inlineStr">
         <is>
-          <t>Triatra + UTPE body &amp; mounting; UT network: 5 site ops, 10 site reps; Italy-made</t>
+          <t>Ferrari stocks units in China (~14 weeks) and parts in Malaysia</t>
         </is>
       </c>
       <c r="Q19" s="37" t="inlineStr">
         <is>
-          <t>Bundle truck + crane + UTPE body + service package; trial-to-buy for key accounts</t>
+          <t>Crane + flatdeck + installation + 2-year warranty; exhibition with Marcom sales kit</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1803,7 @@
       </c>
       <c r="O20" s="37" t="inlineStr">
         <is>
-          <t>China-made; official distributor PT Gaya Makmur Tractors (18 branches)</t>
+          <t>Made in China</t>
         </is>
       </c>
       <c r="P20" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Deck v4: template-exact STP/4P tables, full feature text, full supply chain detail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cx9kswyecF7JAB1Rr5vVcV
</commit_message>
<xml_diff>
--- a/nedp_deck/stp4p/Crane_STP_4P_Medium_Heavy.xlsx
+++ b/nedp_deck/stp4p/Crane_STP_4P_Medium_Heavy.xlsx
@@ -950,16 +950,16 @@
       </c>
       <c r="L5" s="40" t="inlineStr">
         <is>
-          <t>Linkage (Red Power = Articulated Powerlink)
-Power boost (PB = AVPS)
-Electronic control (ECM = EBB)
-Auto fold (Magic Touch = Magic Touch)</t>
+          <t>Linkage: Ferrari Red Power = Amco Veba Articulated Powerlink
+Power boost: Ferrari PB = Amco Veba AVPS
+Electronic control: Ferrari ECM = Amco Veba EBB
+Auto fold: Ferrari Magic Touch = Amco Veba Magic Touch</t>
         </is>
       </c>
       <c r="M5" s="40" t="inlineStr">
         <is>
-          <t>Extension speed (RS)
-Oscillation (SDV)</t>
+          <t>Extension speed: Ferrari RS; Amco Veba: none
+Oscillation: Ferrari SDV (Smooth Descent Valve: less boom flex and dynamic load); Amco Veba: none</t>
         </is>
       </c>
       <c r="N5" s="42" t="n">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="L6" s="43" t="inlineStr">
         <is>
-          <t>Electronic control (Load limiter* = Paltronic 50)</t>
+          <t>Electronic control: XCMG Load limiter* = Sany Palfinger Paltronic 50</t>
         </is>
       </c>
       <c r="M6" s="43" t="inlineStr">
         <is>
-          <t>Parity: wins on price/delivery</t>
+          <t>No extra named feature. Needs a special price to beat Sany Palfinger (now +4%)</t>
         </is>
       </c>
       <c r="N6" s="45" t="n">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="L7" s="40" t="inlineStr">
         <is>
-          <t>Electronic control (Load limiter* = Paltronic 50)</t>
+          <t>Electronic control: XCMG Load limiter* = Sany Palfinger Paltronic 50</t>
         </is>
       </c>
       <c r="M7" s="40" t="inlineStr">
         <is>
-          <t>Parity: wins on price/delivery</t>
+          <t>No extra named feature. Wins on price: −9% vs Sany Palfinger</t>
         </is>
       </c>
       <c r="N7" s="42" t="n">
@@ -1173,16 +1173,16 @@
       </c>
       <c r="L8" s="46" t="inlineStr">
         <is>
-          <t>Power boost (PB = HPLS (MH))
-Extension speed (RS = High speed ext. (ROU))
-Electronic control (ECM = Paltronic 50)</t>
+          <t>Power boost: Ferrari PB = Sany Palfinger HPLS (MH)
+Extension speed: Ferrari RS = Sany Palfinger High speed ext. (ROU)
+Electronic control: Ferrari ECM = Sany Palfinger Paltronic 50</t>
         </is>
       </c>
       <c r="M8" s="46" t="inlineStr">
         <is>
-          <t>Linkage (Red Power)
-Oscillation (SDV)
-Auto fold (Magic Touch)</t>
+          <t>Linkage: Ferrari Red Power; Sany Palfinger: none
+Oscillation: Ferrari SDV (Smooth Descent Valve: less boom flex and dynamic load); Sany Palfinger: none
+Auto fold: Ferrari Magic Touch (opens and stows the crane automatically); Sany Palfinger: none</t>
         </is>
       </c>
       <c r="N8" s="48" t="n">
@@ -1405,16 +1405,16 @@
       </c>
       <c r="L15" s="40" t="inlineStr">
         <is>
-          <t>Linkage (Red Power = Articulated Powerlink)
-Power boost (PB = AVPS)
-Electronic control (ECM = EBB)
-Auto fold (Magic Touch = Magic Touch)</t>
+          <t>Linkage: Ferrari Red Power = Amco Veba Articulated Powerlink
+Power boost: Ferrari PB = Amco Veba AVPS
+Electronic control: Ferrari ECM = Amco Veba EBB
+Auto fold: Ferrari Magic Touch = Amco Veba Magic Touch</t>
         </is>
       </c>
       <c r="M15" s="40" t="inlineStr">
         <is>
-          <t>Extension speed (RS)
-Oscillation (SDV)</t>
+          <t>Extension speed: Ferrari RS; Amco Veba: none
+Oscillation: Ferrari SDV (Smooth Descent Valve: less boom flex and dynamic load); Amco Veba: none</t>
         </is>
       </c>
       <c r="N15" s="42" t="n">
@@ -1482,12 +1482,17 @@
       </c>
       <c r="L16" s="46" t="inlineStr">
         <is>
-          <t>All 6 named features equal (linkage, power boost, extension speed, oscillation, electronic control, auto fold)</t>
+          <t>Linkage: Ferrari Red Power = Palfinger Power Link Plus
+Power boost: Ferrari PB = Palfinger HPLS
+Extension speed: Ferrari RS = Palfinger High Speed Extension
+Oscillation: Ferrari SDV = Palfinger AOS
+Electronic control: Ferrari ECM = Palfinger PALTRONIC 150
+Auto fold: Ferrari Magic Touch = Palfinger P-Fold</t>
         </is>
       </c>
       <c r="M16" s="46" t="inlineStr">
         <is>
-          <t>Parity: wins on price/delivery</t>
+          <t>No extra named feature. Wins on delivery: stock in China (~14 weeks) vs Palfinger built in Europe</t>
         </is>
       </c>
       <c r="N16" s="48" t="n">
@@ -1557,16 +1562,16 @@
       </c>
       <c r="L17" s="40" t="inlineStr">
         <is>
-          <t>Power boost (PB = HPLS (MH))
-Extension speed (RS = High speed ext. (ROU))
-Electronic control (ECM = Paltronic 50)</t>
+          <t>Power boost: Ferrari PB = Sany Palfinger HPLS (MH)
+Extension speed: Ferrari RS = Sany Palfinger High speed ext. (ROU)
+Electronic control: Ferrari ECM = Sany Palfinger Paltronic 50</t>
         </is>
       </c>
       <c r="M17" s="40" t="inlineStr">
         <is>
-          <t>Linkage (Red Power)
-Oscillation (SDV)
-Auto fold (Magic Touch)</t>
+          <t>Linkage: Ferrari Red Power; Sany Palfinger: none
+Oscillation: Ferrari SDV (Smooth Descent Valve: less boom flex and dynamic load); Sany Palfinger: none
+Auto fold: Ferrari Magic Touch (opens and stows the crane automatically); Sany Palfinger: none</t>
         </is>
       </c>
       <c r="N17" s="42" t="inlineStr">
@@ -1636,12 +1641,17 @@
       </c>
       <c r="L18" s="46" t="inlineStr">
         <is>
-          <t>All 6 named features equal (linkage, power boost, extension speed, oscillation, electronic control, auto fold)</t>
+          <t>Linkage: Ferrari Red Power = Palfinger Power Link Plus
+Power boost: Ferrari PB = Palfinger HPLS
+Extension speed: Ferrari RS = Palfinger High Speed Extension
+Oscillation: Ferrari SDV = Palfinger AOS
+Electronic control: Ferrari ECM = Palfinger PALTRONIC 150
+Auto fold: Ferrari Magic Touch = Palfinger P-Fold</t>
         </is>
       </c>
       <c r="M18" s="46" t="inlineStr">
         <is>
-          <t>Parity: wins on price/delivery</t>
+          <t>No extra named feature. Wins on delivery: stock in China (~14 weeks) vs Palfinger built in Europe</t>
         </is>
       </c>
       <c r="N18" s="48" t="n">
@@ -1711,12 +1721,17 @@
       </c>
       <c r="L19" s="40" t="inlineStr">
         <is>
-          <t>All 6 named features equal (linkage, power boost, extension speed, oscillation, electronic control, auto fold)</t>
+          <t>Linkage: Ferrari Red Power = Palfinger Power Link Plus
+Power boost: Ferrari PB = Palfinger HPLS
+Extension speed: Ferrari RS = Palfinger High Speed Extension
+Oscillation: Ferrari SDV = Palfinger AOS
+Electronic control: Ferrari ECM = Palfinger PALTRONIC 150
+Auto fold: Ferrari Magic Touch = Palfinger P-Fold</t>
         </is>
       </c>
       <c r="M19" s="40" t="inlineStr">
         <is>
-          <t>Parity: wins on price/delivery</t>
+          <t>No extra named feature. Wins on delivery: stock in China (~14 weeks) vs Palfinger built in Europe</t>
         </is>
       </c>
       <c r="N19" s="42" t="inlineStr">

</xml_diff>